<commit_message>
Daily slate 2026-05-29 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-27.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-27.xlsx
@@ -474,13 +474,13 @@
         <v>165</v>
       </c>
       <c r="E2" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G2" t="n">
-        <v>50.3</v>
+        <v>50.9</v>
       </c>
     </row>
     <row r="3">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E4" t="n">
         <v>16</v>
       </c>
       <c r="F4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G4" t="n">
-        <v>48.5</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E5" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F5" t="n">
         <v>36</v>
       </c>
       <c r="G5" t="n">
-        <v>47.1</v>
+        <v>47.8</v>
       </c>
     </row>
     <row r="6">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="E11" t="n">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="F11" t="n">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G11" t="n">
-        <v>60.1</v>
+        <v>60.3</v>
       </c>
     </row>
     <row r="12">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E14" t="n">
         <v>52</v>
       </c>
       <c r="F14" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G14" t="n">
-        <v>25.7</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="E15" t="n">
         <v>102</v>
       </c>
       <c r="F15" t="n">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="G15" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="16">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3335</v>
+        <v>3355</v>
       </c>
       <c r="E17" t="n">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="F17" t="n">
-        <v>2715</v>
+        <v>2734</v>
       </c>
       <c r="G17" t="n">
-        <v>18.6</v>
+        <v>18.5</v>
       </c>
     </row>
   </sheetData>
@@ -1342,7 +1342,7 @@
         <v>17</v>
       </c>
       <c r="R4" t="n">
-        <v>60.8</v>
+        <v>62.7</v>
       </c>
       <c r="S4" t="n">
         <v>51</v>
@@ -1576,10 +1576,10 @@
         <v>137</v>
       </c>
       <c r="D7" t="n">
-        <v>60.1</v>
+        <v>60.3</v>
       </c>
       <c r="E7" t="n">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="F7" t="n">
         <v>62.4</v>
@@ -1594,16 +1594,16 @@
         <v>388</v>
       </c>
       <c r="J7" t="n">
-        <v>25.7</v>
+        <v>25.5</v>
       </c>
       <c r="K7" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="L7" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="M7" t="n">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="N7" t="n">
         <v>25.7</v>
@@ -1612,22 +1612,22 @@
         <v>183</v>
       </c>
       <c r="P7" t="n">
-        <v>18.6</v>
+        <v>18.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>3335</v>
+        <v>3355</v>
       </c>
       <c r="R7" t="n">
-        <v>50.3</v>
+        <v>50.9</v>
       </c>
       <c r="S7" t="n">
         <v>165</v>
       </c>
       <c r="T7" t="n">
-        <v>48.5</v>
+        <v>47.1</v>
       </c>
       <c r="U7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="V7" t="n">
         <v>52.1</v>
@@ -1648,10 +1648,10 @@
         <v>284</v>
       </c>
       <c r="AB7" t="n">
-        <v>47.1</v>
+        <v>47.8</v>
       </c>
       <c r="AC7" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AD7" t="n">
         <v>50</v>

</xml_diff>